<commit_message>
5 Company Project Complete
</commit_message>
<xml_diff>
--- a/data/processed/aapl_info.xlsx
+++ b/data/processed/aapl_info.xlsx
@@ -8,10 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Apple Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Apple Forecasting" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Apple Valuation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Apple Ratios" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Apple Charts" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Apple Charts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Apple Forecasting" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Apple Valuation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Apple Ratios" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -101,16 +101,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -194,291 +185,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Apple Revenue Forecast (Avg Growth Rate)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <layout>
-        <manualLayout>
-          <xMode val="edge"/>
-          <yMode val="edge"/>
-          <wMode val="factor"/>
-          <hMode val="factor"/>
-          <x val="0.12"/>
-          <y val="0.2"/>
-          <w val="0.82"/>
-          <h val="0.68"/>
-        </manualLayout>
-      </layout>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Apple Forecasting'!B1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln w="22000">
-              <a:solidFill>
-                <a:srgbClr val="1F77B4"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="circle"/>
-            <size val="7"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="1F77B4"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="1F77B4"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Apple Forecasting'!$A$2:$A$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Apple Forecasting'!$B$2:$B$7</f>
-            </numRef>
-          </val>
-          <smooth val="0"/>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Fiscal Year</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Revenue ($ Billions)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Apple Revenue Forecast (Linear Trend)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <layout>
-        <manualLayout>
-          <xMode val="edge"/>
-          <yMode val="edge"/>
-          <wMode val="factor"/>
-          <hMode val="factor"/>
-          <x val="0.12"/>
-          <y val="0.2"/>
-          <w val="0.82"/>
-          <h val="0.68"/>
-        </manualLayout>
-      </layout>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'Apple Forecasting'!C1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln w="22000">
-              <a:solidFill>
-                <a:srgbClr val="D62728"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="circle"/>
-            <size val="7"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="D62728"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="D62728"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Apple Forecasting'!$A$2:$A$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Apple Forecasting'!$C$2:$C$7</f>
-            </numRef>
-          </val>
-          <smooth val="0"/>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Fiscal Year</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Revenue ($ Billions)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -648,9 +354,8 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -791,9 +496,8 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -934,9 +638,8 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -1077,56 +780,291 @@
 </chartSpace>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7200000" cy="3600000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>19</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7200000" cy="3600000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Apple Revenue Forecast (Avg Growth Rate)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.12"/>
+          <y val="0.2"/>
+          <w val="0.82"/>
+          <h val="0.68"/>
+        </manualLayout>
+      </layout>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Apple Forecasting'!B1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="1F77B4"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="7"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F77B4"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1F77B4"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Apple Forecasting'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Apple Forecasting'!$B$2:$B$7</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Fiscal Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Revenue ($ Billions)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Apple Revenue Forecast (Linear Trend)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <layout>
+        <manualLayout>
+          <xMode val="edge"/>
+          <yMode val="edge"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.12"/>
+          <y val="0.2"/>
+          <w val="0.82"/>
+          <h val="0.68"/>
+        </manualLayout>
+      </layout>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Apple Forecasting'!C1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="D62728"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="7"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="D62728"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="D62728"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Apple Forecasting'!$A$2:$A$7</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Apple Forecasting'!$C$2:$C$7</f>
+            </numRef>
+          </val>
+          <smooth val="0"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Fiscal Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="0"/>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Revenue ($ Billions)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1219,6 +1157,55 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7200000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AAPLSummary" displayName="AAPLSummary" ref="A1:F7" headerRowCount="1">
   <autoFilter ref="A1:F7"/>
@@ -1252,7 +1239,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="AAPLRatios" displayName="AAPLRatios" ref="A1:E7" headerRowCount="1">
   <autoFilter ref="A1:E7"/>
   <tableColumns count="5">
-    <tableColumn id="1" name="Apple Financial Ratios"/>
+    <tableColumn id="1" name="Ratios for Apple Inc."/>
     <tableColumn id="2" name="2022"/>
     <tableColumn id="3" name="2023"/>
     <tableColumn id="4" name="2024"/>
@@ -1733,17 +1720,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>2025 Value</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
@@ -1841,13 +1828,13 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Overall Score</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr"/>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="B17" s="7" t="n"/>
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>6.5/10</t>
         </is>
@@ -1867,7 +1854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1878,12 +1865,22 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Avg Growth Forecast</t>
+          <t>Revenue</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Linear Trend Forecast</t>
+          <t>net_income</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>diluted_eps</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>stock_price</t>
         </is>
       </c>
     </row>
@@ -1892,10 +1889,16 @@
         <v>2022</v>
       </c>
       <c r="B2" t="n">
-        <v>394.3</v>
+        <v>394.328</v>
       </c>
       <c r="C2" t="n">
-        <v>394.3</v>
+        <v>99.803</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6.11</v>
+      </c>
+      <c r="E2" t="n">
+        <v>150.43</v>
       </c>
     </row>
     <row r="3">
@@ -1903,10 +1906,16 @@
         <v>2023</v>
       </c>
       <c r="B3" t="n">
-        <v>383.3</v>
+        <v>383.285</v>
       </c>
       <c r="C3" t="n">
-        <v>383.3</v>
+        <v>96.995</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6.13</v>
+      </c>
+      <c r="E3" t="n">
+        <v>171.21</v>
       </c>
     </row>
     <row r="4">
@@ -1914,10 +1923,16 @@
         <v>2024</v>
       </c>
       <c r="B4" t="n">
-        <v>391</v>
+        <v>391.035</v>
       </c>
       <c r="C4" t="n">
-        <v>391</v>
+        <v>93.736</v>
+      </c>
+      <c r="D4" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="E4" t="n">
+        <v>227.79</v>
       </c>
     </row>
     <row r="5">
@@ -1925,32 +1940,16 @@
         <v>2025</v>
       </c>
       <c r="B5" t="n">
-        <v>416.2</v>
+        <v>416.161</v>
       </c>
       <c r="C5" t="n">
-        <v>416.2</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>2026</v>
-      </c>
-      <c r="B6" t="n">
-        <v>424</v>
-      </c>
-      <c r="C6" t="n">
-        <v>414.5</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>2027</v>
-      </c>
-      <c r="B7" t="n">
-        <v>432</v>
-      </c>
-      <c r="C7" t="n">
-        <v>421.8</v>
+        <v>112.01</v>
+      </c>
+      <c r="D5" t="n">
+        <v>7.46</v>
+      </c>
+      <c r="E5" t="n">
+        <v>255.46</v>
       </c>
     </row>
   </sheetData>
@@ -1960,6 +1959,104 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Fiscal Year</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Avg Growth Forecast</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Linear Trend Forecast</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B2" t="n">
+        <v>394.3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>394.3</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B3" t="n">
+        <v>383.3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>383.3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B4" t="n">
+        <v>391</v>
+      </c>
+      <c r="C4" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B5" t="n">
+        <v>416.2</v>
+      </c>
+      <c r="C5" t="n">
+        <v>416.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B6" t="n">
+        <v>424</v>
+      </c>
+      <c r="C6" t="n">
+        <v>414.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2027</v>
+      </c>
+      <c r="B7" t="n">
+        <v>432</v>
+      </c>
+      <c r="C7" t="n">
+        <v>421.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2086,7 +2183,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2105,7 +2202,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Apple Financial Ratios</t>
+          <t>Ratios for Apple Inc.</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -2249,114 +2346,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Fiscal Year</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>net_income</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>diluted_eps</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>stock_price</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B2" t="n">
-        <v>394.328</v>
-      </c>
-      <c r="C2" t="n">
-        <v>99.803</v>
-      </c>
-      <c r="D2" t="n">
-        <v>6.11</v>
-      </c>
-      <c r="E2" t="n">
-        <v>150.43</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B3" t="n">
-        <v>383.285</v>
-      </c>
-      <c r="C3" t="n">
-        <v>96.995</v>
-      </c>
-      <c r="D3" t="n">
-        <v>6.13</v>
-      </c>
-      <c r="E3" t="n">
-        <v>171.21</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B4" t="n">
-        <v>391.035</v>
-      </c>
-      <c r="C4" t="n">
-        <v>93.736</v>
-      </c>
-      <c r="D4" t="n">
-        <v>6.08</v>
-      </c>
-      <c r="E4" t="n">
-        <v>227.79</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B5" t="n">
-        <v>416.161</v>
-      </c>
-      <c r="C5" t="n">
-        <v>112.01</v>
-      </c>
-      <c r="D5" t="n">
-        <v>7.46</v>
-      </c>
-      <c r="E5" t="n">
-        <v>255.46</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>